<commit_message>
Vérification du questionnaire (en cours) : réponses actives, répartitions à refaire, bornes, relecture des questions
Une réponse devenue inapplicable reste en base mais ne compte plus (conditions,
calcul, avancement, total pré-rempli). Une répartition dont une ligne a été
ajoutée ou retirée ne compte plus tant que le total n'est pas de nouveau juste,
sans redistribution. Bornes sur les champs chiffrés, total de COM-12.01 sur ses
trois colonnes, D27 et D13 lus dans RH-08.01 et RH-28.01, 29 questions
reformulées. Inventaire, matrice des dépendances et plan du contrôle navigateur
dans docs/verification (travail en cours, journal dans progression.md).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VuMzauPSe4mKhw7WeK1nNo
</commit_message>
<xml_diff>
--- a/CAXE_Banque_Questions.xlsx
+++ b/CAXE_Banque_Questions.xlsx
@@ -754,7 +754,7 @@
       </c>
       <c r="S1" s="4" t="inlineStr">
         <is>
-          <t>Total imposé (Colonne = valeur)</t>
+          <t>Total imposé (Colonne = valeur ; plusieurs colonnes séparées par « ; »)</t>
         </is>
       </c>
       <c r="T1" s="3" t="inlineStr">
@@ -870,7 +870,7 @@
       <c r="H3" s="5" t="n"/>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de votre chiffre d'affaires vient de chacune de ces catégories de clients ?</t>
+          <t>Sur les 12 derniers mois, quelle part de votre chiffre d'affaires vient de chacune de ces catégories de clients ?</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
@@ -968,7 +968,7 @@
       <c r="P4" s="7" t="n"/>
       <c r="Q4" s="6" t="inlineStr">
         <is>
-          <t>Clients sur 12 mois [nombre]</t>
+          <t>Clients sur 12 mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R4" s="6" t="inlineStr">
@@ -1042,7 +1042,7 @@
       <c r="P5" s="7" t="n"/>
       <c r="Q5" s="6" t="inlineStr">
         <is>
-          <t>Fois par an [nombre]</t>
+          <t>Fois par an [nombre 0-]</t>
         </is>
       </c>
       <c r="R5" s="6" t="inlineStr">
@@ -1170,7 +1170,7 @@
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>À quelle distance de votre entreprise se trouvent vos clients ?</t>
+          <t>Sur les 12 derniers mois, à quelle distance de votre entreprise se trouvaient vos clients ?</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -1312,7 +1312,7 @@
       <c r="H9" s="5" t="n"/>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de votre chiffre d'affaires faites-vous dans cette zone ?</t>
+          <t>Sur les 12 derniers mois, quelle part de votre chiffre d'affaires avez-vous faite dans cette zone ?</t>
         </is>
       </c>
       <c r="J9" s="7" t="n"/>
@@ -1446,7 +1446,7 @@
       <c r="H11" s="5" t="n"/>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de vos ventes se fait hors de votre région, y compris à l'étranger ?</t>
+          <t>Sur les 12 derniers mois, quelle part de vos commandes vient de clients situés hors de votre région, y compris à l'étranger ?</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Cochez tous ceux qui vous ont amené au moins un client. Bouche-à-oreille : vos clients et votre entourage. Partenaires : des professionnels qui vous recommandent. Réseaux sociaux : vos publications ; leur publicité payante va dans Publicité en ligne. Emailing et SMS : vos messages à vos propres contacts ; à des inconnus, c'est de la Prospection. Plateformes : TheFork, Doctolib, Booking, Uber Eats, Malt, marketplace… Annuaires : PagesJaunes et sites d'annuaires. Réseaux d'affaires : BNI, CCI, clubs d'entrepreneurs. Réseau ou enseigne : les clients envoyés par votre franchise ou votre groupement. Passage : les clients qui passent devant chez vous.</t>
+          <t>Cochez tous ceux qui vous ont amené au moins un client : chaque canal coché ouvre ensuite quelques questions sur lui (part des demandes, des nouveaux clients, du chiffre d'affaires). Bouche-à-oreille : vos clients et votre entourage. Partenaires : des professionnels qui vous recommandent. Réseaux sociaux : vos publications ; leur publicité payante va dans Publicité en ligne. Emailing et SMS : vos messages à vos propres contacts ; à des inconnus, c'est de la Prospection. Plateformes : TheFork, Doctolib, Booking, Uber Eats, Malt, marketplace… Annuaires : PagesJaunes et sites d'annuaires. Réseaux d'affaires : BNI, CCI, clubs d'entrepreneurs. Réseau ou enseigne : les clients envoyés par votre franchise ou votre groupement. Passage : les clients qui passent devant chez vous.</t>
         </is>
       </c>
       <c r="K17" s="7" t="n"/>
@@ -1930,12 +1930,12 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de vos {demandes} vient de chaque canal ?</t>
+          <t>Sur les 12 derniers mois, quelle part de vos {demandes} est arrivée par chaque canal ?</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Par exemple : 50 % bouche-à-oreille, 30 % fiche Google, 20 % site internet. Une estimation suffit.</t>
+          <t>Une demande compte dans un seul canal : celui par lequel elle vous est arrivée. Par exemple : 50 % bouche-à-oreille, 30 % fiche Google, 20 % site internet. Une estimation suffit.</t>
         </is>
       </c>
       <c r="K18" s="7" t="n"/>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de vos nouveaux clients vient de chaque canal ?</t>
+          <t>Sur les 12 derniers mois, quelle part de vos nouveaux clients est arrivée par chaque canal ?</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
@@ -2420,7 +2420,7 @@
       <c r="P24" s="7" t="n"/>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>Par semaine [nombre]</t>
+          <t>Par semaine [nombre 0-]</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
@@ -2926,7 +2926,7 @@
       <c r="P31" s="7" t="n"/>
       <c r="Q31" s="6" t="inlineStr">
         <is>
-          <t>Contacts apportés par mois (moyenne des 3 derniers mois) [nombre] · Nouveaux clients sur 12 mois [nombre] · Chiffre d'affaires sur 12 mois [€ 0-]</t>
+          <t>Contacts apportés par mois (moyenne des 3 derniers mois) [nombre 0-] · Nouveaux clients sur 12 mois [nombre 0-] · Chiffre d'affaires sur 12 mois [€ 0-]</t>
         </is>
       </c>
       <c r="R31" s="6" t="inlineStr">
@@ -3078,7 +3078,7 @@
       <c r="P33" s="7" t="n"/>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>Avis au total [nombre] · Note sur 5 [nombre 0-5] · Avis reçus sur les 6 derniers mois [nombre]</t>
+          <t>Avis au total [nombre 0-] · Note sur 5 [nombre 0-5] · Avis reçus sur les 6 derniers mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R33" s="7" t="n"/>
@@ -3152,7 +3152,7 @@
       <c r="P34" s="7" t="n"/>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>Vues de votre fiche [nombre] · Appels [nombre] · Demandes d'itinéraire [nombre] · Clics vers votre site [nombre]</t>
+          <t>Vues de votre fiche [nombre 0-] · Appels [nombre 0-] · Demandes d'itinéraire [nombre 0-] · Clics vers votre site [nombre 0-]</t>
         </is>
       </c>
       <c r="R34" s="7" t="n"/>
@@ -3226,7 +3226,7 @@
       <c r="P35" s="7" t="n"/>
       <c r="Q35" s="6" t="inlineStr">
         <is>
-          <t>Nom [texte] · Avis [nombre] · Note sur 5 [nombre 0-5]</t>
+          <t>Nom [texte] · Avis [nombre 0-] · Note sur 5 [nombre 0-5]</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -3376,7 +3376,7 @@
       <c r="P37" s="7" t="n"/>
       <c r="Q37" s="6" t="inlineStr">
         <is>
-          <t>Note [nombre] · Note sur [choix: 5 / 10] · Nombre d'avis [nombre]</t>
+          <t>Note [nombre 0-] · Note sur [choix: 5 / 10] · Nombre d'avis [nombre 0-]</t>
         </is>
       </c>
       <c r="R37" s="7" t="n"/>
@@ -3526,7 +3526,7 @@
       <c r="P39" s="7" t="n"/>
       <c r="Q39" s="6" t="inlineStr">
         <is>
-          <t>Nombre de recherches [nombre]</t>
+          <t>Nombre de recherches [nombre 0-]</t>
         </is>
       </c>
       <c r="R39" s="6" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>Pour chaque plateforme, quelle part de votre chiffre d'affaires vous apporte-t-elle, et quel pourcentage prélève-t-elle ?</t>
+          <t>Sur les 12 derniers mois, pour chaque plateforme : quelle part de votre chiffre d'affaires vous a-t-elle apportée, et quel pourcentage prélève-t-elle ?</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
@@ -3961,8 +3961,12 @@
           <t>%</t>
         </is>
       </c>
-      <c r="N45" s="7" t="n"/>
-      <c r="O45" s="7" t="n"/>
+      <c r="N45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="6" t="n">
+        <v>100</v>
+      </c>
       <c r="P45" s="7" t="n"/>
       <c r="Q45" s="7" t="n"/>
       <c r="R45" s="7" t="n"/>
@@ -4239,7 +4243,7 @@
       <c r="O49" s="7" t="n"/>
       <c r="P49" s="6" t="inlineStr">
         <is>
-          <t>Téléphone · Email · Formulaire du site · Messages (réseaux sociaux, WhatsApp, SMS)</t>
+          <t>Téléphone · Email · Formulaire du site · Messages (réseaux sociaux, WhatsApp, SMS) · Aucun : je réponds aussi vite partout</t>
         </is>
       </c>
       <c r="Q49" s="7" t="n"/>
@@ -4452,7 +4456,7 @@
       <c r="P52" s="7" t="n"/>
       <c r="Q52" s="6" t="inlineStr">
         <is>
-          <t>Annulés en vous prévenant [nombre] · Absents sans prévenir [nombre]</t>
+          <t>Annulés en vous prévenant [nombre 0-] · Absents sans prévenir [nombre 0-]</t>
         </is>
       </c>
       <c r="R52" s="7" t="n"/>
@@ -4742,7 +4746,7 @@
       <c r="P56" s="7" t="n"/>
       <c r="Q56" s="6" t="inlineStr">
         <is>
-          <t>Nombre par mois [nombre] · Montant total par mois [€ 0-]</t>
+          <t>Nombre par mois [nombre 0-] · Montant total par mois [€ 0-]</t>
         </is>
       </c>
       <c r="R56" s="7" t="n"/>
@@ -4816,7 +4820,7 @@
       <c r="P57" s="7" t="n"/>
       <c r="Q57" s="6" t="inlineStr">
         <is>
-          <t>Nombre par mois [nombre] · Montant total par mois [€ 0-]</t>
+          <t>Nombre par mois [nombre 0-] · Montant total par mois [€ 0-]</t>
         </is>
       </c>
       <c r="R57" s="7" t="n"/>
@@ -5104,7 +5108,7 @@
       <c r="P61" s="7" t="n"/>
       <c r="Q61" s="6" t="inlineStr">
         <is>
-          <t>Nombre [nombre] · Montant total [€ 0-]</t>
+          <t>Nombre [nombre 0-] · Montant total [€ 0-]</t>
         </is>
       </c>
       <c r="R61" s="7" t="n"/>
@@ -5567,7 +5571,7 @@
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>Répartissez, par exemple 50 % prix, 30 % pas assez relancé, 20 % projet abandonné. Une estimation suffit.</t>
+          <t>Comptez chaque affaire perdue une fois, avec sa raison principale. Répartissez, par exemple 50 % prix, 30 % pas assez relancé, 20 % projet abandonné. Une estimation suffit.</t>
         </is>
       </c>
       <c r="K68" s="7" t="n"/>
@@ -5724,7 +5728,7 @@
       <c r="P70" s="7" t="n"/>
       <c r="Q70" s="6" t="inlineStr">
         <is>
-          <t>Couverts par service [nombre]</t>
+          <t>Couverts par service [nombre 0-]</t>
         </is>
       </c>
       <c r="R70" s="6" t="inlineStr">
@@ -6116,7 +6120,7 @@
       <c r="H76" s="5" t="n"/>
       <c r="I76" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de votre chiffre d'affaires vient de la vente à emporter et de la livraison ?</t>
+          <t>Sur les 12 derniers mois, quelle part de votre chiffre d'affaires vient de la vente à emporter et de la livraison ?</t>
         </is>
       </c>
       <c r="J76" s="7" t="n"/>
@@ -6784,7 +6788,7 @@
       <c r="H86" s="5" t="n"/>
       <c r="I86" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de votre chiffre d'affaires vient de ce que vous vendez en plus : {hors_location} ?</t>
+          <t>Sur les 12 derniers mois, quelle part de votre chiffre d'affaires vient de ce que vous vendez en plus : {hors_location} ?</t>
         </is>
       </c>
       <c r="J86" s="7" t="n"/>
@@ -6869,8 +6873,12 @@
           <t>%</t>
         </is>
       </c>
-      <c r="N87" s="7" t="n"/>
-      <c r="O87" s="7" t="n"/>
+      <c r="N87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O87" s="6" t="n">
+        <v>100</v>
+      </c>
       <c r="P87" s="7" t="n"/>
       <c r="Q87" s="7" t="n"/>
       <c r="R87" s="7" t="n"/>
@@ -7150,7 +7158,7 @@
       <c r="P91" s="7" t="n"/>
       <c r="Q91" s="6" t="inlineStr">
         <is>
-          <t>Nombre [nombre] · Montant estimé [€ 0-]</t>
+          <t>Nombre [nombre 0-] · Montant estimé [€ 0-]</t>
         </is>
       </c>
       <c r="R91" s="7" t="n"/>
@@ -7342,7 +7350,7 @@
       <c r="H94" s="5" t="n"/>
       <c r="I94" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de votre chiffre d'affaires fait chacune de ces offres ?</t>
+          <t>Sur les 12 derniers mois, quelle part de votre chiffre d'affaires a fait chacune de ces offres ?</t>
         </is>
       </c>
       <c r="J94" s="6" t="inlineStr">
@@ -9228,12 +9236,12 @@
       <c r="H121" s="5" t="n"/>
       <c r="I121" s="6" t="inlineStr">
         <is>
-          <t>Parmi vos clients de l'an dernier, quelle part vous a de nouveau choisi cette année ?</t>
+          <t>Parmi vos clients de l'année d'avant, quelle part vous a de nouveau choisi sur les 12 derniers mois ?</t>
         </is>
       </c>
       <c r="J121" s="6" t="inlineStr">
         <is>
-          <t>Une estimation suffit. Si vous ne connaissez pas vos clients par leur nom, estimez la part d'habitués.</t>
+          <t>L'année d'avant : les 12 mois qui précèdent les 12 derniers mois. Une estimation suffit. Si vous ne connaissez pas vos clients par leur nom, estimez la part d'habitués.</t>
         </is>
       </c>
       <c r="K121" s="7" t="n"/>
@@ -9722,7 +9730,7 @@
       <c r="P128" s="7" t="n"/>
       <c r="Q128" s="6" t="inlineStr">
         <is>
-          <t>Clients sous contrat ou abonnés [nombre] · Total payé par mois [€ 0-]</t>
+          <t>Clients sous contrat ou abonnés [nombre 0-] · Total payé par mois [€ 0-]</t>
         </is>
       </c>
       <c r="R128" s="7" t="n"/>
@@ -9788,7 +9796,7 @@
       <c r="P129" s="7" t="n"/>
       <c r="Q129" s="6" t="inlineStr">
         <is>
-          <t>Clients sous contrat ou abonnés [nombre] · Total payé par mois [€ 0-]</t>
+          <t>Clients sous contrat ou abonnés [nombre 0-] · Total payé par mois [€ 0-]</t>
         </is>
       </c>
       <c r="R129" s="6" t="inlineStr">
@@ -10227,7 +10235,11 @@
           <t>À quel moment demandez-vous à vos clients de vous recommander ?</t>
         </is>
       </c>
-      <c r="J136" s="7" t="n"/>
+      <c r="J136" s="6" t="inlineStr">
+        <is>
+          <t>Si vous le faites à plusieurs moments, choisissez le plus fréquent.</t>
+        </is>
+      </c>
       <c r="K136" s="7" t="n"/>
       <c r="L136" s="6" t="inlineStr">
         <is>
@@ -11138,7 +11150,7 @@
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="6" t="inlineStr">
         <is>
-          <t>Personnes [nombre] · Dont à temps partiel [nombre]</t>
+          <t>Personnes [nombre 0-] · Dont à temps partiel [nombre 0-]</t>
         </is>
       </c>
       <c r="R149" s="6" t="inlineStr">
@@ -11352,7 +11364,7 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="6" t="inlineStr">
         <is>
-          <t>Heures travaillées [heures] · Heures facturées [heures]</t>
+          <t>Heures travaillées [heures 0-] · Heures facturées [heures 0-]</t>
         </is>
       </c>
       <c r="R152" s="7" t="n"/>
@@ -11554,7 +11566,7 @@
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="6" t="inlineStr">
         <is>
-          <t>Heures d'ouverture [heures]</t>
+          <t>Heures d'ouverture [heures 0-]</t>
         </is>
       </c>
       <c r="R155" s="6" t="inlineStr">
@@ -11986,7 +11998,7 @@
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="6" t="inlineStr">
         <is>
-          <t>Clients perdus par mois [nombre]</t>
+          <t>Clients perdus par mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R161" s="6" t="inlineStr">
@@ -12266,7 +12278,7 @@
       <c r="P165" s="7" t="n"/>
       <c r="Q165" s="6" t="inlineStr">
         <is>
-          <t>Nombre [nombre]</t>
+          <t>Nombre [nombre 0-]</t>
         </is>
       </c>
       <c r="R165" s="6" t="inlineStr">
@@ -12340,7 +12352,7 @@
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="6" t="inlineStr">
         <is>
-          <t>Heures par semaine [heures] · Budget par mois [€ 0-]</t>
+          <t>Heures par semaine [heures 0-] · Budget par mois [€ 0-]</t>
         </is>
       </c>
       <c r="R166" s="7" t="n"/>
@@ -12410,7 +12422,7 @@
       <c r="P167" s="7" t="n"/>
       <c r="Q167" s="6" t="inlineStr">
         <is>
-          <t>Courses [nombre] · Heures disponibles [heures] · Heures avec un client ou un colis [heures]</t>
+          <t>Courses [nombre 0-] · Heures disponibles [heures 0-] · Heures avec un client ou un colis [heures 0-]</t>
         </is>
       </c>
       <c r="R167" s="7" t="n"/>
@@ -12480,7 +12492,7 @@
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="6" t="inlineStr">
         <is>
-          <t>Kilomètres au total [km] · Dont avec un client ou un colis [km]</t>
+          <t>Kilomètres au total [km 0-] · Dont avec un client ou un colis [km 0-]</t>
         </is>
       </c>
       <c r="R168" s="7" t="n"/>
@@ -12545,7 +12557,9 @@
           <t>nombre</t>
         </is>
       </c>
-      <c r="N169" s="7" t="n"/>
+      <c r="N169" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="O169" s="7" t="n"/>
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="n"/>
@@ -12611,8 +12625,12 @@
           <t>%</t>
         </is>
       </c>
-      <c r="N170" s="7" t="n"/>
-      <c r="O170" s="7" t="n"/>
+      <c r="N170" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O170" s="6" t="n">
+        <v>100</v>
+      </c>
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="n"/>
       <c r="R170" s="7" t="n"/>
@@ -12673,8 +12691,12 @@
           <t>%</t>
         </is>
       </c>
-      <c r="N171" s="7" t="n"/>
-      <c r="O171" s="7" t="n"/>
+      <c r="N171" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O171" s="6" t="n">
+        <v>100</v>
+      </c>
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="n"/>
       <c r="R171" s="7" t="n"/>
@@ -12880,7 +12902,7 @@
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="6" t="inlineStr">
         <is>
-          <t>Votre délai [jours] · Délai des concurrents [jours]</t>
+          <t>Votre délai [jours 0-] · Délai des concurrents [jours 0-]</t>
         </is>
       </c>
       <c r="R174" s="7" t="n"/>
@@ -12950,7 +12972,7 @@
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="6" t="inlineStr">
         <is>
-          <t>Biens en stock [nombre] · Jours en stock en moyenne [jours]</t>
+          <t>Biens en stock [nombre 0-] · Jours en stock en moyenne [jours 0-]</t>
         </is>
       </c>
       <c r="R175" s="7" t="n"/>
@@ -13019,8 +13041,12 @@
           <t>%</t>
         </is>
       </c>
-      <c r="N176" s="7" t="n"/>
-      <c r="O176" s="7" t="n"/>
+      <c r="N176" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O176" s="6" t="n">
+        <v>100</v>
+      </c>
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="n"/>
       <c r="R176" s="7" t="n"/>
@@ -13151,7 +13177,9 @@
           <t>nombre</t>
         </is>
       </c>
-      <c r="N178" s="7" t="n"/>
+      <c r="N178" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="O178" s="7" t="n"/>
       <c r="P178" s="7" t="n"/>
       <c r="Q178" s="7" t="n"/>
@@ -13214,7 +13242,7 @@
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="6" t="inlineStr">
         <is>
-          <t>Mandats [nombre] · Dont exclusifs [nombre]</t>
+          <t>Mandats [nombre 0-] · Dont exclusifs [nombre 0-]</t>
         </is>
       </c>
       <c r="R179" s="7" t="n"/>
@@ -13279,7 +13307,9 @@
           <t>jours</t>
         </is>
       </c>
-      <c r="N180" s="7" t="n"/>
+      <c r="N180" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="O180" s="7" t="n"/>
       <c r="P180" s="7" t="n"/>
       <c r="Q180" s="7" t="n"/>
@@ -13345,8 +13375,12 @@
           <t>%</t>
         </is>
       </c>
-      <c r="N181" s="7" t="n"/>
-      <c r="O181" s="7" t="n"/>
+      <c r="N181" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O181" s="6" t="n">
+        <v>100</v>
+      </c>
       <c r="P181" s="7" t="n"/>
       <c r="Q181" s="7" t="n"/>
       <c r="R181" s="7" t="n"/>
@@ -13407,7 +13441,9 @@
           <t>nombre</t>
         </is>
       </c>
-      <c r="N182" s="7" t="n"/>
+      <c r="N182" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="O182" s="7" t="n"/>
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="n"/>
@@ -13602,7 +13638,7 @@
       <c r="H185" s="5" t="n"/>
       <c r="I185" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de votre chiffre d'affaires fait chacune de ces offres ?</t>
+          <t>Sur les 12 derniers mois, quelle part de votre chiffre d'affaires a fait chacune de ces offres ?</t>
         </is>
       </c>
       <c r="J185" s="6" t="inlineStr">
@@ -13774,7 +13810,7 @@
       <c r="P187" s="7" t="n"/>
       <c r="Q187" s="6" t="inlineStr">
         <is>
-          <t>Heures par mois [heures]</t>
+          <t>Heures par mois [heures 0-]</t>
         </is>
       </c>
       <c r="R187" s="6" t="inlineStr">
@@ -14404,7 +14440,7 @@
       <c r="P196" s="7" t="n"/>
       <c r="Q196" s="6" t="inlineStr">
         <is>
-          <t>Clients sous contrat ou abonnés [nombre] · Total payé par mois [€ 0-]</t>
+          <t>Clients sous contrat ou abonnés [nombre 0-] · Total payé par mois [€ 0-]</t>
         </is>
       </c>
       <c r="R196" s="7" t="n"/>
@@ -14894,7 +14930,7 @@
       <c r="P203" s="7" t="n"/>
       <c r="Q203" s="6" t="inlineStr">
         <is>
-          <t>Heures travaillées [heures] · Heures facturées [heures]</t>
+          <t>Heures travaillées [heures 0-] · Heures facturées [heures 0-]</t>
         </is>
       </c>
       <c r="R203" s="7" t="n"/>
@@ -15034,7 +15070,7 @@
       <c r="P205" s="7" t="n"/>
       <c r="Q205" s="6" t="inlineStr">
         <is>
-          <t>Heures [heures] · Coût [€ 0-]</t>
+          <t>Heures [heures 0-] · Coût [€ 0-]</t>
         </is>
       </c>
       <c r="R205" s="7" t="n"/>
@@ -15592,7 +15628,7 @@
       <c r="P213" s="7" t="n"/>
       <c r="Q213" s="6" t="inlineStr">
         <is>
-          <t>Coût par mois [€ 0-] · Utilisateurs [nombre] · Renouvellement [mois et année] · Résiliation [choix: À tout moment / Durée minimum à respecter] · Utilisation [choix: Utilisé / Peu utilisé / Pas utilisé]</t>
+          <t>Coût par mois [€ 0-] · Utilisateurs [nombre 0-] · Renouvellement [mois et année] · Résiliation [choix: À tout moment / Durée minimum à respecter] · Utilisation [choix: Utilisé / Peu utilisé / Pas utilisé]</t>
         </is>
       </c>
       <c r="R213" s="6" t="inlineStr">
@@ -15866,7 +15902,7 @@
       <c r="P217" s="7" t="n"/>
       <c r="Q217" s="6" t="inlineStr">
         <is>
-          <t>Reprises par mois [nombre] · Retours par mois [nombre] · Gestes commerciaux par mois [nombre] · Coût moyen d'une reprise [€ 0-] · Coût moyen d'un geste commercial [€ 0-]</t>
+          <t>Reprises par mois [nombre 0-] · Retours par mois [nombre 0-] · Gestes commerciaux par mois [nombre 0-] · Coût moyen d'une reprise [€ 0-] · Coût moyen d'un geste commercial [€ 0-]</t>
         </is>
       </c>
       <c r="R217" s="7" t="n"/>
@@ -16776,7 +16812,7 @@
       <c r="P230" s="7" t="n"/>
       <c r="Q230" s="6" t="inlineStr">
         <is>
-          <t>Montant [€ 0-] · Mois pour vous en remettre [mois]</t>
+          <t>Montant [€ 0-] · Mois pour vous en remettre [mois 0-]</t>
         </is>
       </c>
       <c r="R230" s="7" t="n"/>
@@ -17066,7 +17102,7 @@
       <c r="P234" s="7" t="n"/>
       <c r="Q234" s="6" t="inlineStr">
         <is>
-          <t>Nombre [nombre] · Montant [€ 0-]</t>
+          <t>Nombre [nombre 0-] · Montant [€ 0-]</t>
         </is>
       </c>
       <c r="R234" s="7" t="n"/>
@@ -17192,7 +17228,7 @@
       </c>
       <c r="I236" s="6" t="inlineStr">
         <is>
-          <t>En réalité, en combien de temps vos clients vous paient-ils ?</t>
+          <t>Sur les 12 derniers mois, en combien de temps vos clients vous ont-ils payé en réalité ?</t>
         </is>
       </c>
       <c r="J236" s="6" t="inlineStr">
@@ -17290,7 +17326,7 @@
       <c r="P237" s="7" t="n"/>
       <c r="Q237" s="6" t="inlineStr">
         <is>
-          <t>Délai réel de paiement [jours]</t>
+          <t>Délai réel de paiement [jours 0-]</t>
         </is>
       </c>
       <c r="R237" s="6" t="inlineStr">
@@ -17722,7 +17758,7 @@
       <c r="P243" s="7" t="n"/>
       <c r="Q243" s="6" t="inlineStr">
         <is>
-          <t>Jours avant la première relance [jours] · Méthode [choix: Toujours, par écrit / Au cas par cas / Aucune relance]</t>
+          <t>Jours avant la première relance [jours 0-] · Méthode [choix: Toujours, par écrit / Au cas par cas / Aucune relance]</t>
         </is>
       </c>
       <c r="R243" s="7" t="n"/>
@@ -17792,7 +17828,7 @@
       <c r="P244" s="7" t="n"/>
       <c r="Q244" s="6" t="inlineStr">
         <is>
-          <t>Nombre de factures [nombre] · Montant [€ 0-]</t>
+          <t>Nombre de factures [nombre 0-] · Montant [€ 0-]</t>
         </is>
       </c>
       <c r="R244" s="7" t="n"/>
@@ -19076,7 +19112,7 @@
       <c r="P262" s="7" t="n"/>
       <c r="Q262" s="6" t="inlineStr">
         <is>
-          <t>Objet [texte] · Prix d'achat [€ 0-] · Installation et frais annexes [€ 0-] · Coûts récurrents par mois [€ 0-] · Mise en service [mois et année] · Durée d'utilisation prévue [ans]</t>
+          <t>Objet [texte] · Prix d'achat [€ 0-] · Installation et frais annexes [€ 0-] · Coûts récurrents par mois [€ 0-] · Mise en service [mois et année] · Durée d'utilisation prévue [ans 0-]</t>
         </is>
       </c>
       <c r="R262" s="7" t="n"/>
@@ -19222,7 +19258,7 @@
       <c r="P264" s="7" t="n"/>
       <c r="Q264" s="6" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires en plus [€ 0-] · Économies de charges [€ 0-] · Heures gagnées [heures]</t>
+          <t>Chiffre d'affaires en plus [€ 0-] · Économies de charges [€ 0-] · Heures gagnées [heures 0-]</t>
         </is>
       </c>
       <c r="R264" s="7" t="n"/>
@@ -19296,7 +19332,7 @@
       <c r="P265" s="7" t="n"/>
       <c r="Q265" s="6" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires en plus [€ 0-] · Économies de charges [€ 0-] · Heures gagnées [heures]</t>
+          <t>Chiffre d'affaires en plus [€ 0-] · Économies de charges [€ 0-] · Heures gagnées [heures 0-]</t>
         </is>
       </c>
       <c r="R265" s="7" t="n"/>
@@ -19772,7 +19808,7 @@
       <c r="P272" s="7" t="n"/>
       <c r="Q272" s="6" t="inlineStr">
         <is>
-          <t>Heures par mois [heures] · Qui [choix: Vous / Un salarié / Le comptable / Un prestataire]</t>
+          <t>Heures par mois [heures 0-] · Qui [choix: Vous / Un salarié / Le comptable / Un prestataire]</t>
         </is>
       </c>
       <c r="R272" s="7" t="n"/>
@@ -20634,7 +20670,7 @@
       <c r="P284" s="7" t="n"/>
       <c r="Q284" s="6" t="inlineStr">
         <is>
-          <t>Ruptures par mois [nombre] · Durée moyenne [jours]</t>
+          <t>Ruptures par mois [nombre 0-] · Durée moyenne [jours 0-]</t>
         </is>
       </c>
       <c r="R284" s="7" t="n"/>
@@ -20708,7 +20744,7 @@
       <c r="P285" s="7" t="n"/>
       <c r="Q285" s="6" t="inlineStr">
         <is>
-          <t>Clients perdus par mois [nombre] · Commandes reportées par mois [nombre]</t>
+          <t>Clients perdus par mois [nombre 0-] · Commandes reportées par mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R285" s="7" t="n"/>
@@ -20778,7 +20814,7 @@
       <c r="P286" s="7" t="n"/>
       <c r="Q286" s="6" t="inlineStr">
         <is>
-          <t>Commandes par mois [nombre] · Méthode [choix: Un seuil de commande pour chaque produit / Un seuil pour les principaux produits / À l'instinct]</t>
+          <t>Commandes par mois [nombre 0-] · Méthode [choix: Un seuil de commande pour chaque produit / Un seuil pour les principaux produits / À l'instinct]</t>
         </is>
       </c>
       <c r="R286" s="7" t="n"/>
@@ -20920,7 +20956,7 @@
       <c r="P288" s="7" t="n"/>
       <c r="Q288" s="6" t="inlineStr">
         <is>
-          <t>Fournisseurs avec un minimum [nombre] · Part du stock achetée seulement pour atteindre ce minimum [% 0-100] · Remise obtenue grâce au volume [% 0-100]</t>
+          <t>Fournisseurs avec un minimum [nombre 0-] · Part du stock achetée seulement pour atteindre ce minimum [% 0-100] · Remise obtenue grâce au volume [% 0-100]</t>
         </is>
       </c>
       <c r="R288" s="7" t="n"/>
@@ -20990,7 +21026,7 @@
       <c r="P289" s="7" t="n"/>
       <c r="Q289" s="6" t="inlineStr">
         <is>
-          <t>Inventaires par an [nombre] · Dernier inventaire [mois et année] · Outil [choix: Aucun / Tableur / Logiciel relié à la caisse]</t>
+          <t>Inventaires par an [nombre 0-] · Dernier inventaire [mois et année] · Outil [choix: Aucun / Tableur / Logiciel relié à la caisse]</t>
         </is>
       </c>
       <c r="R289" s="7" t="n"/>
@@ -21134,7 +21170,7 @@
       <c r="P291" s="7" t="n"/>
       <c r="Q291" s="6" t="inlineStr">
         <is>
-          <t>Écart à l'inventaire précédent [€ 0-] · Corrections à la main par mois (moyenne des 3 derniers mois) [nombre]</t>
+          <t>Écart à l'inventaire précédent [€ 0-] · Corrections à la main par mois (moyenne des 3 derniers mois) [nombre 0-]</t>
         </is>
       </c>
       <c r="R291" s="7" t="n"/>
@@ -21806,7 +21842,7 @@
       <c r="P301" s="7" t="n"/>
       <c r="Q301" s="6" t="inlineStr">
         <is>
-          <t>Heures par mois [heures]</t>
+          <t>Heures par mois [heures 0-]</t>
         </is>
       </c>
       <c r="R301" s="6" t="inlineStr">
@@ -22558,7 +22594,7 @@
       <c r="P312" s="7" t="n"/>
       <c r="Q312" s="6" t="inlineStr">
         <is>
-          <t>Jours [jours] · Heures [heures]</t>
+          <t>Jours [jours 0-] · Heures [heures 0-]</t>
         </is>
       </c>
       <c r="R312" s="7" t="n"/>
@@ -23164,7 +23200,7 @@
       <c r="P321" s="7" t="n"/>
       <c r="Q321" s="6" t="inlineStr">
         <is>
-          <t>Heures [heures] · Coût [€ 0-]</t>
+          <t>Heures [heures 0-] · Coût [€ 0-]</t>
         </is>
       </c>
       <c r="R321" s="7" t="n"/>
@@ -23504,7 +23540,7 @@
       <c r="P326" s="7" t="n"/>
       <c r="Q326" s="6" t="inlineStr">
         <is>
-          <t>Heures en plus par semaine [heures]</t>
+          <t>Heures en plus par semaine [heures 0-]</t>
         </is>
       </c>
       <c r="R326" s="6" t="inlineStr">
@@ -24759,7 +24795,7 @@
       <c r="O345" s="7" t="n"/>
       <c r="P345" s="6" t="inlineStr">
         <is>
-          <t>Intérim ou extras · Heures supplémentaires · Rien de particulier</t>
+          <t>Intérim ou extras · Heures supplémentaires · Rien de particulier · Les deux</t>
         </is>
       </c>
       <c r="Q345" s="7" t="n"/>
@@ -24830,7 +24866,7 @@
       <c r="P346" s="7" t="n"/>
       <c r="Q346" s="6" t="inlineStr">
         <is>
-          <t>Tâches clés [nombre] · Dont décrites par écrit [nombre]</t>
+          <t>Tâches clés [nombre 0-] · Dont décrites par écrit [nombre 0-]</t>
         </is>
       </c>
       <c r="R346" s="7" t="n"/>
@@ -25302,7 +25338,7 @@
       <c r="P353" s="7" t="n"/>
       <c r="Q353" s="6" t="inlineStr">
         <is>
-          <t>Reprises par mois [nombre] · Temps moyen d'une reprise [heures]</t>
+          <t>Reprises par mois [nombre 0-] · Temps moyen d'une reprise [heures 0-]</t>
         </is>
       </c>
       <c r="R353" s="7" t="n"/>
@@ -25442,7 +25478,7 @@
       <c r="P355" s="7" t="n"/>
       <c r="Q355" s="6" t="inlineStr">
         <is>
-          <t>Corrections mineures [nombre] · Reprises complètes [nombre]</t>
+          <t>Corrections mineures [nombre 0-] · Reprises complètes [nombre 0-]</t>
         </is>
       </c>
       <c r="R355" s="7" t="n"/>
@@ -25582,7 +25618,7 @@
       <c r="P357" s="7" t="n"/>
       <c r="Q357" s="6" t="inlineStr">
         <is>
-          <t>Laquelle [texte] · Heures par semaine [heures] · Qui la fait [texte] · Outil utilisé [texte]</t>
+          <t>Laquelle [texte] · Heures par semaine [heures 0-] · Qui la fait [texte] · Outil utilisé [texte]</t>
         </is>
       </c>
       <c r="R357" s="6" t="inlineStr">
@@ -25784,7 +25820,7 @@
       <c r="P360" s="7" t="n"/>
       <c r="Q360" s="6" t="inlineStr">
         <is>
-          <t>Réunions par mois [nombre] · Durée moyenne en minutes [nombre] · Participants en moyenne [nombre]</t>
+          <t>Réunions par mois [nombre 0-] · Durée moyenne en minutes [nombre 0-] · Participants en moyenne [nombre 0-]</t>
         </is>
       </c>
       <c r="R360" s="7" t="n"/>
@@ -26188,7 +26224,7 @@
       <c r="P366" s="7" t="n"/>
       <c r="Q366" s="6" t="inlineStr">
         <is>
-          <t>Moyen prévu [oui / non] · Idées appliquées sur 6 mois [nombre]</t>
+          <t>Moyen prévu [oui / non] · Idées appliquées sur 6 mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R366" s="7" t="n"/>
@@ -26398,7 +26434,7 @@
       <c r="P369" s="7" t="n"/>
       <c r="Q369" s="6" t="inlineStr">
         <is>
-          <t>Jours de formation [jours] · Transmission organisée entre collègues [oui / non]</t>
+          <t>Jours de formation [jours 0-] · Transmission organisée entre collègues [oui / non]</t>
         </is>
       </c>
       <c r="R369" s="7" t="n"/>
@@ -26878,7 +26914,7 @@
       <c r="P376" s="7" t="n"/>
       <c r="Q376" s="6" t="inlineStr">
         <is>
-          <t>Candidatures par poste [nombre] · Entretiens par poste [nombre] · Candidats qui ont refusé l'offre [nombre]</t>
+          <t>Candidatures par poste [nombre 0-] · Entretiens par poste [nombre 0-] · Candidats qui ont refusé l'offre [nombre 0-]</t>
         </is>
       </c>
       <c r="R376" s="7" t="n"/>
@@ -26952,7 +26988,7 @@
       <c r="P377" s="7" t="n"/>
       <c r="Q377" s="6" t="inlineStr">
         <is>
-          <t>Coût d'un recrutement [€ 0-] · Heures passées par vous et votre équipe [heures]</t>
+          <t>Coût d'un recrutement [€ 0-] · Heures passées par vous et votre équipe [heures 0-]</t>
         </is>
       </c>
       <c r="R377" s="7" t="n"/>
@@ -27508,7 +27544,7 @@
       <c r="P385" s="7" t="n"/>
       <c r="Q385" s="6" t="inlineStr">
         <is>
-          <t>Poste [texte] · Semaines pour le maîtriser [semaines]</t>
+          <t>Poste [texte] · Semaines pour le maîtriser [semaines 0-]</t>
         </is>
       </c>
       <c r="R385" s="7" t="n"/>
@@ -27574,7 +27610,7 @@
       <c r="P386" s="7" t="n"/>
       <c r="Q386" s="6" t="inlineStr">
         <is>
-          <t>Départs [nombre]</t>
+          <t>Départs [nombre 0-]</t>
         </is>
       </c>
       <c r="R386" s="6" t="inlineStr">
@@ -27644,7 +27680,7 @@
       <c r="P387" s="7" t="n"/>
       <c r="Q387" s="6" t="inlineStr">
         <is>
-          <t>Départs sur un poste clé [nombre] · Remplacement [choix: Fait / En cours / Non]</t>
+          <t>Départs sur un poste clé [nombre 0-] · Remplacement [choix: Fait / En cours / Non]</t>
         </is>
       </c>
       <c r="R387" s="7" t="n"/>
@@ -27784,7 +27820,7 @@
       <c r="P389" s="7" t="n"/>
       <c r="Q389" s="6" t="inlineStr">
         <is>
-          <t>Poste le plus concerné [texte] · Ancienneté moyenne au départ [mois]</t>
+          <t>Poste le plus concerné [texte] · Ancienneté moyenne au départ [mois 0-]</t>
         </is>
       </c>
       <c r="R389" s="7" t="n"/>
@@ -27920,7 +27956,7 @@
       <c r="P391" s="7" t="n"/>
       <c r="Q391" s="6" t="inlineStr">
         <is>
-          <t>À l'initiative de la recrue [nombre] · À votre initiative [nombre]</t>
+          <t>À l'initiative de la recrue [nombre 0-] · À votre initiative [nombre 0-]</t>
         </is>
       </c>
       <c r="R391" s="6" t="inlineStr">
@@ -28404,7 +28440,7 @@
       <c r="P398" s="7" t="n"/>
       <c r="Q398" s="6" t="inlineStr">
         <is>
-          <t>Semaines pour former un remplaçant [semaines]</t>
+          <t>Semaines pour former un remplaçant [semaines 0-]</t>
         </is>
       </c>
       <c r="R398" s="6" t="inlineStr">
@@ -28621,7 +28657,7 @@
       <c r="O401" s="7" t="n"/>
       <c r="P401" s="6" t="inlineStr">
         <is>
-          <t>Préparés avec l'équipe · Annoncés · Imposés</t>
+          <t>Préparés avec l'équipe · Annoncés · Imposés · Aucun changement récent</t>
         </is>
       </c>
       <c r="Q401" s="7" t="n"/>
@@ -28972,7 +29008,7 @@
       <c r="P406" s="7" t="n"/>
       <c r="Q406" s="6" t="inlineStr">
         <is>
-          <t>Heures par semaine [heures] · S'apprend en moins d'un mois [oui / non] · Méthode écrite [oui / non]</t>
+          <t>Heures par semaine [heures 0-] · S'apprend en moins d'un mois [oui / non] · Méthode écrite [oui / non]</t>
         </is>
       </c>
       <c r="R406" s="6" t="inlineStr">
@@ -29186,7 +29222,7 @@
       <c r="P409" s="7" t="n"/>
       <c r="Q409" s="6" t="inlineStr">
         <is>
-          <t>Clients perdus par mois [nombre]</t>
+          <t>Clients perdus par mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R409" s="6" t="inlineStr">
@@ -29748,7 +29784,7 @@
       <c r="P417" s="7" t="n"/>
       <c r="Q417" s="6" t="inlineStr">
         <is>
-          <t>Personnes [nombre] · Dont à temps partiel [nombre]</t>
+          <t>Personnes [nombre 0-] · Dont à temps partiel [nombre 0-]</t>
         </is>
       </c>
       <c r="R417" s="6" t="inlineStr">
@@ -29822,7 +29858,7 @@
       <c r="P418" s="7" t="n"/>
       <c r="Q418" s="6" t="inlineStr">
         <is>
-          <t>Personnes [nombre]</t>
+          <t>Personnes [nombre 0-]</t>
         </is>
       </c>
       <c r="R418" s="6" t="inlineStr">
@@ -29892,7 +29928,7 @@
       <c r="P419" s="7" t="n"/>
       <c r="Q419" s="6" t="inlineStr">
         <is>
-          <t>Qui le fait [choix: Vous / Un responsable / Chacun s'organise / Il n'y a pas de planning] · Heures par semaine [heures]</t>
+          <t>Qui le fait [choix: Vous / Un responsable / Chacun s'organise / Il n'y a pas de planning] · Heures par semaine [heures 0-]</t>
         </is>
       </c>
       <c r="R419" s="7" t="n"/>
@@ -30230,7 +30266,7 @@
       <c r="P424" s="7" t="n"/>
       <c r="Q424" s="6" t="inlineStr">
         <is>
-          <t>Responsables, vous non compris [nombre] · Personnes suivies par un responsable, au plus [nombre]</t>
+          <t>Responsables, vous non compris [nombre 0-] · Personnes suivies par un responsable, au plus [nombre 0-]</t>
         </is>
       </c>
       <c r="R424" s="7" t="n"/>
@@ -30419,7 +30455,7 @@
       </c>
       <c r="J427" s="6" t="inlineStr">
         <is>
-          <t>Cochez une catégorie, deux au plus.</t>
+          <t>Répondez « Oui » pour une catégorie, deux au plus.</t>
         </is>
       </c>
       <c r="K427" s="7" t="n"/>
@@ -30914,7 +30950,7 @@
       <c r="P434" s="7" t="n"/>
       <c r="Q434" s="6" t="inlineStr">
         <is>
-          <t>Disponibles [nombre] · Publiées sur le site [nombre] · Publiées sur les réseaux [nombre]</t>
+          <t>Disponibles [nombre 0-] · Publiées sur le site [nombre 0-] · Publiées sur les réseaux [nombre 0-]</t>
         </is>
       </c>
       <c r="R434" s="6" t="inlineStr">
@@ -31186,7 +31222,7 @@
       <c r="P438" s="7" t="n"/>
       <c r="Q438" s="6" t="inlineStr">
         <is>
-          <t>Ouverture du compte [mois et année] · Publications par mois (moyenne des 3 derniers mois) [nombre] · Format principal [choix: Vidéo courte / Vidéo longue / Carrousel / Photo / Texte / Story] · Dernière publication [mois et année] · Qui publie [choix: Vous / Un salarié / Un prestataire]</t>
+          <t>Ouverture du compte [mois et année] · Publications par mois (moyenne des 3 derniers mois) [nombre 0-] · Format principal [choix: Vidéo courte / Vidéo longue / Carrousel / Photo / Texte / Story] · Dernière publication [mois et année] · Qui publie [choix: Vous / Un salarié / Un prestataire]</t>
         </is>
       </c>
       <c r="R438" s="6" t="inlineStr">
@@ -31590,12 +31626,12 @@
       <c r="H444" s="5" t="n"/>
       <c r="I444" s="6" t="inlineStr">
         <is>
-          <t>Quelle part de vos demandes, de vos nouveaux clients et de votre chiffre d'affaires vient de chaque canal ?</t>
+          <t>Sur les 12 derniers mois, quelle part de vos demandes, de vos nouveaux clients et de votre chiffre d'affaires est arrivée par chaque canal ?</t>
         </is>
       </c>
       <c r="J444" s="6" t="inlineStr">
         <is>
-          <t>Une ligne par canal coché. Si l'agent Acquisition a déjà posé ces questions, les réponses sont reprises.</t>
+          <t>Une ligne par canal coché. Chaque colonne fait 100 % : une demande, un client ou un euro ne compte que dans un canal, celui par lequel il est arrivé. Si l'agent Acquisition a déjà posé ces questions, les réponses sont reprises.</t>
         </is>
       </c>
       <c r="K444" s="7" t="n"/>
@@ -31620,7 +31656,7 @@
       </c>
       <c r="S444" s="6" t="inlineStr">
         <is>
-          <t>Part des demandes = 100</t>
+          <t>Part des demandes ; Part des nouveaux clients ; Part du chiffre d'affaires sur 12 mois = 100</t>
         </is>
       </c>
       <c r="T444" s="5" t="inlineStr">
@@ -31834,7 +31870,7 @@
       <c r="P447" s="7" t="n"/>
       <c r="Q447" s="6" t="inlineStr">
         <is>
-          <t>Par mois [nombre]</t>
+          <t>Par mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R447" s="6" t="inlineStr">
@@ -31892,7 +31928,7 @@
       </c>
       <c r="I448" s="6" t="inlineStr">
         <is>
-          <t>D'où viennent les visites de votre site ?</t>
+          <t>Sur les 3 derniers mois, d'où sont venues les visites de votre site ?</t>
         </is>
       </c>
       <c r="J448" s="6" t="inlineStr">
@@ -32338,7 +32374,7 @@
       <c r="P454" s="7" t="n"/>
       <c r="Q454" s="6" t="inlineStr">
         <is>
-          <t>Vues de votre fiche [nombre] · Appels [nombre] · Demandes d'itinéraire [nombre] · Clics vers votre site [nombre]</t>
+          <t>Vues de votre fiche [nombre 0-] · Appels [nombre 0-] · Demandes d'itinéraire [nombre 0-] · Clics vers votre site [nombre 0-]</t>
         </is>
       </c>
       <c r="R454" s="7" t="n"/>
@@ -32412,7 +32448,7 @@
       <c r="P455" s="7" t="n"/>
       <c r="Q455" s="6" t="inlineStr">
         <is>
-          <t>Contacts [nombre]</t>
+          <t>Contacts [nombre 0-]</t>
         </is>
       </c>
       <c r="R455" s="6" t="inlineStr">
@@ -32486,7 +32522,7 @@
       <c r="P456" s="7" t="n"/>
       <c r="Q456" s="6" t="inlineStr">
         <is>
-          <t>Nouveaux contacts par mois [nombre] · Source principale [choix: Site / Offre gratuite / Boutique ou comptoir / Salon ou événement / Réseaux sociaux / Nouveaux clients]</t>
+          <t>Nouveaux contacts par mois [nombre 0-] · Source principale [choix: Site / Offre gratuite / Boutique ou comptoir / Salon ou événement / Réseaux sociaux / Nouveaux clients]</t>
         </is>
       </c>
       <c r="R456" s="7" t="n"/>
@@ -32560,7 +32596,7 @@
       <c r="P457" s="7" t="n"/>
       <c r="Q457" s="6" t="inlineStr">
         <is>
-          <t>Dernier envoi [mois et année] · Envois sur 6 mois [nombre]</t>
+          <t>Dernier envoi [mois et année] · Envois sur 6 mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R457" s="7" t="n"/>
@@ -32630,7 +32666,7 @@
       <c r="P458" s="7" t="n"/>
       <c r="Q458" s="6" t="inlineStr">
         <is>
-          <t>Demandes [nombre] · Clients obtenus [nombre]</t>
+          <t>Demandes [nombre 0-] · Clients obtenus [nombre 0-]</t>
         </is>
       </c>
       <c r="R458" s="7" t="n"/>
@@ -32770,7 +32806,7 @@
       <c r="P460" s="7" t="n"/>
       <c r="Q460" s="6" t="inlineStr">
         <is>
-          <t>Taux d'ouverture [% 0-100] · Taux de clic [% 0-100] · Désinscriptions [nombre] · Réponses [nombre]</t>
+          <t>Taux d'ouverture [% 0-100] · Taux de clic [% 0-100] · Désinscriptions [nombre 0-] · Réponses [nombre 0-]</t>
         </is>
       </c>
       <c r="R460" s="7" t="n"/>
@@ -32980,7 +33016,7 @@
       <c r="P463" s="7" t="n"/>
       <c r="Q463" s="6" t="inlineStr">
         <is>
-          <t>Abonnés [nombre] · Personnes touchées par mois (moyenne des 3 derniers mois) [nombre]</t>
+          <t>Abonnés [nombre 0-] · Personnes touchées par mois (moyenne des 3 derniers mois) [nombre 0-]</t>
         </is>
       </c>
       <c r="R463" s="6" t="inlineStr">
@@ -33054,7 +33090,7 @@
       <c r="P464" s="7" t="n"/>
       <c r="Q464" s="6" t="inlineStr">
         <is>
-          <t>Nouveaux abonnés [nombre] · Désabonnements [nombre]</t>
+          <t>Nouveaux abonnés [nombre 0-] · Désabonnements [nombre 0-]</t>
         </is>
       </c>
       <c r="R464" s="6" t="inlineStr">
@@ -33112,7 +33148,7 @@
       </c>
       <c r="I465" s="6" t="inlineStr">
         <is>
-          <t>Sur chaque réseau, quelle part des personnes touchées ne vous suit pas encore ?</t>
+          <t>Sur les 3 derniers mois, quelle part des personnes touchées sur chaque réseau ne vous suivait pas encore ?</t>
         </is>
       </c>
       <c r="J465" s="6" t="inlineStr">
@@ -33210,7 +33246,7 @@
       <c r="P466" s="7" t="n"/>
       <c r="Q466" s="6" t="inlineStr">
         <is>
-          <t>J'aime [nombre] · Commentaires [nombre] · Partages [nombre] · Enregistrements [nombre]</t>
+          <t>J'aime [nombre 0-] · Commentaires [nombre 0-] · Partages [nombre 0-] · Enregistrements [nombre 0-]</t>
         </is>
       </c>
       <c r="R466" s="6" t="inlineStr">
@@ -33288,7 +33324,7 @@
       <c r="P467" s="7" t="n"/>
       <c r="Q467" s="6" t="inlineStr">
         <is>
-          <t>Clics par mois [nombre] · Destination principale [choix: Site / Fiche Google / Formulaire / Prise de rendez-vous / Téléphone / WhatsApp / Email / Page produit ou offre]</t>
+          <t>Clics par mois [nombre 0-] · Destination principale [choix: Site / Fiche Google / Formulaire / Prise de rendez-vous / Téléphone / WhatsApp / Email / Page produit ou offre]</t>
         </is>
       </c>
       <c r="R467" s="6" t="inlineStr">
@@ -33432,7 +33468,7 @@
       <c r="P469" s="7" t="n"/>
       <c r="Q469" s="6" t="inlineStr">
         <is>
-          <t>Visiteurs de la page de l'offre [nombre] · Contacts récoltés [nombre] · Contacts vraiment intéressés [nombre] · Rendez-vous obtenus [nombre] · Nouveaux clients [nombre]</t>
+          <t>Visiteurs de la page de l'offre [nombre 0-] · Contacts récoltés [nombre 0-] · Contacts vraiment intéressés [nombre 0-] · Rendez-vous obtenus [nombre 0-] · Nouveaux clients [nombre 0-]</t>
         </is>
       </c>
       <c r="R469" s="7" t="n"/>
@@ -33702,12 +33738,12 @@
       </c>
       <c r="I473" s="6" t="inlineStr">
         <is>
-          <t>Parmi les clients et les demandes qui vous viennent des réseaux sociaux, quelle part vient de chaque réseau ?</t>
+          <t>Sur les 12 derniers mois, parmi les demandes qui vous sont venues des réseaux sociaux, quelle part est venue de chaque réseau ?</t>
         </is>
       </c>
       <c r="J473" s="6" t="inlineStr">
         <is>
-          <t>Une estimation suffit. Leur nombre total est déjà demandé avec vos canaux : ici, on le répartit entre vos réseaux.</t>
+          <t>Une estimation suffit. Une demande compte dans un seul réseau : celui par lequel elle est arrivée. Leur nombre total est déjà demandé avec vos canaux : ici, on le répartit entre vos réseaux.</t>
         </is>
       </c>
       <c r="K473" s="7" t="n"/>
@@ -33800,7 +33836,7 @@
       <c r="P474" s="7" t="n"/>
       <c r="Q474" s="6" t="inlineStr">
         <is>
-          <t>Messages par mois [nombre] · Dont demandes commerciales [nombre] · Dont service après-vente [nombre]</t>
+          <t>Messages par mois [nombre 0-] · Dont demandes commerciales [nombre 0-] · Dont service après-vente [nombre 0-]</t>
         </is>
       </c>
       <c r="R474" s="6" t="inlineStr">
@@ -33956,7 +33992,7 @@
       <c r="P476" s="7" t="n"/>
       <c r="Q476" s="6" t="inlineStr">
         <is>
-          <t>Rendez-vous ou devis [nombre] · Nouveaux clients [nombre]</t>
+          <t>Rendez-vous ou devis [nombre 0-] · Nouveaux clients [nombre 0-]</t>
         </is>
       </c>
       <c r="R476" s="7" t="n"/>
@@ -34160,7 +34196,7 @@
       <c r="P479" s="7" t="n"/>
       <c r="Q479" s="6" t="inlineStr">
         <is>
-          <t>Publications [nombre]</t>
+          <t>Publications [nombre 0-]</t>
         </is>
       </c>
       <c r="R479" s="6" t="inlineStr">
@@ -34450,7 +34486,7 @@
       <c r="P483" s="7" t="n"/>
       <c r="Q483" s="6" t="inlineStr">
         <is>
-          <t>Heures par semaine [heures]</t>
+          <t>Heures par semaine [heures 0-]</t>
         </is>
       </c>
       <c r="R483" s="6" t="inlineStr">
@@ -34974,7 +35010,7 @@
       <c r="P490" s="7" t="n"/>
       <c r="Q490" s="6" t="inlineStr">
         <is>
-          <t>Semaines avec une publication [nombre 0-12] · Plus longue pause [semaines]</t>
+          <t>Semaines avec une publication [nombre 0-12] · Plus longue pause [semaines 0-]</t>
         </is>
       </c>
       <c r="R490" s="6" t="inlineStr">
@@ -35194,7 +35230,7 @@
       <c r="P493" s="7" t="n"/>
       <c r="Q493" s="6" t="inlineStr">
         <is>
-          <t>Prêts ou programmés [nombre] · À finaliser [nombre] · Idées notées [nombre]</t>
+          <t>Prêts ou programmés [nombre 0-] · À finaliser [nombre 0-] · Idées notées [nombre 0-]</t>
         </is>
       </c>
       <c r="R493" s="7" t="n"/>
@@ -35264,7 +35300,7 @@
       <c r="P494" s="7" t="n"/>
       <c r="Q494" s="6" t="inlineStr">
         <is>
-          <t>Autres photos et vidéos utilisables : équipe, coulisses, lieu [nombre] · Modèles de visuels [oui / non] · Contenus intemporels à republier [nombre]</t>
+          <t>Autres photos et vidéos utilisables : équipe, coulisses, lieu [nombre 0-] · Modèles de visuels [oui / non] · Contenus intemporels à republier [nombre 0-]</t>
         </is>
       </c>
       <c r="R494" s="7" t="n"/>
@@ -35338,7 +35374,7 @@
       <c r="P495" s="7" t="n"/>
       <c r="Q495" s="6" t="inlineStr">
         <is>
-          <t>Abonnés il y a 6 mois [nombre]</t>
+          <t>Abonnés il y a 6 mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R495" s="6" t="inlineStr">
@@ -35416,7 +35452,7 @@
       <c r="P496" s="7" t="n"/>
       <c r="Q496" s="6" t="inlineStr">
         <is>
-          <t>Réseau [texte] · Personnes touchées [nombre] · Réactions [nombre] · Visites du profil [nombre] · Nouveaux abonnés [nombre] · Clics [nombre] · Messages ou demandes [nombre]</t>
+          <t>Réseau [texte] · Personnes touchées [nombre 0-] · Réactions [nombre 0-] · Visites du profil [nombre 0-] · Nouveaux abonnés [nombre 0-] · Clics [nombre 0-] · Messages ou demandes [nombre 0-]</t>
         </is>
       </c>
       <c r="R496" s="6" t="inlineStr">
@@ -35474,7 +35510,7 @@
       </c>
       <c r="I497" s="6" t="inlineStr">
         <is>
-          <t>Pour chacune de ces 6 publications, quel est son texte et son lien ?</t>
+          <t>Pour vos 3 meilleures et vos 3 moins bonnes publications des 3 derniers mois, quel est leur texte et leur lien ?</t>
         </is>
       </c>
       <c r="J497" s="6" t="inlineStr">
@@ -35568,7 +35604,7 @@
       <c r="P498" s="7" t="n"/>
       <c r="Q498" s="6" t="inlineStr">
         <is>
-          <t>Vues par vidéo [nombre] · Secondes regardées en moyenne [nombre] · Part vue jusqu'au bout [% 0-100]</t>
+          <t>Vues par vidéo [nombre 0-] · Secondes regardées en moyenne [nombre 0-] · Part vue jusqu'au bout [% 0-100]</t>
         </is>
       </c>
       <c r="R498" s="7" t="n"/>
@@ -35968,7 +36004,7 @@
       <c r="P504" s="7" t="n"/>
       <c r="Q504" s="6" t="inlineStr">
         <is>
-          <t>Avis au total [nombre] · Note sur 5 [nombre 0-5] · Avis reçus sur les 6 derniers mois [nombre]</t>
+          <t>Avis au total [nombre 0-] · Note sur 5 [nombre 0-5] · Avis reçus sur les 6 derniers mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R504" s="7" t="n"/>
@@ -36038,7 +36074,7 @@
       <c r="P505" s="7" t="n"/>
       <c r="Q505" s="6" t="inlineStr">
         <is>
-          <t>Avis [nombre] · Note sur 5 [nombre 0-5]</t>
+          <t>Avis [nombre 0-] · Note sur 5 [nombre 0-5]</t>
         </is>
       </c>
       <c r="R505" s="6" t="inlineStr">
@@ -36112,7 +36148,7 @@
       <c r="P506" s="7" t="n"/>
       <c r="Q506" s="6" t="inlineStr">
         <is>
-          <t>5 étoiles [nombre] · 4 étoiles [nombre] · 3 étoiles ou moins [nombre]</t>
+          <t>5 étoiles [nombre 0-] · 4 étoiles [nombre 0-] · 3 étoiles ou moins [nombre 0-]</t>
         </is>
       </c>
       <c r="R506" s="7" t="n"/>
@@ -36388,7 +36424,7 @@
       <c r="P510" s="7" t="n"/>
       <c r="Q510" s="6" t="inlineStr">
         <is>
-          <t>Avis positifs avec une réponse [% 0-100] · Avis négatifs avec une réponse [% 0-100] · Délai moyen de réponse [jours]</t>
+          <t>Avis positifs avec une réponse [% 0-100] · Avis négatifs avec une réponse [% 0-100] · Délai moyen de réponse [jours 0-]</t>
         </is>
       </c>
       <c r="R510" s="7" t="n"/>
@@ -36590,7 +36626,7 @@
       <c r="P513" s="7" t="n"/>
       <c r="Q513" s="6" t="inlineStr">
         <is>
-          <t>Presse [nombre] · Associations ou réseaux locaux [nombre] · Créateurs de contenu [nombre] · Autres entreprises [nombre]</t>
+          <t>Presse [nombre 0-] · Associations ou réseaux locaux [nombre 0-] · Créateurs de contenu [nombre 0-] · Autres entreprises [nombre 0-]</t>
         </is>
       </c>
       <c r="R513" s="7" t="n"/>
@@ -36660,7 +36696,7 @@
       <c r="P514" s="7" t="n"/>
       <c r="Q514" s="6" t="inlineStr">
         <is>
-          <t>Collaborations [nombre] · Ventes suivies [nombre]</t>
+          <t>Collaborations [nombre 0-] · Ventes suivies [nombre 0-]</t>
         </is>
       </c>
       <c r="R514" s="7" t="n"/>
@@ -38308,7 +38344,7 @@
       <c r="P537" s="7" t="n"/>
       <c r="Q537" s="6" t="inlineStr">
         <is>
-          <t>Visites du profil par mois [nombre]</t>
+          <t>Visites du profil par mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R537" s="6" t="inlineStr">
@@ -38608,7 +38644,7 @@
       <c r="P541" s="7" t="n"/>
       <c r="Q541" s="6" t="inlineStr">
         <is>
-          <t>Personnes contactées par mois [nombre] · Devenues clientes par mois [nombre]</t>
+          <t>Personnes contactées par mois [nombre 0-] · Devenues clientes par mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R541" s="7" t="n"/>
@@ -38748,7 +38784,7 @@
       <c r="P543" s="7" t="n"/>
       <c r="Q543" s="6" t="inlineStr">
         <is>
-          <t>Apparitions [nombre] · Clics [nombre] · Position moyenne [nombre 1-100]</t>
+          <t>Apparitions [nombre 0-] · Clics [nombre 0-] · Position moyenne [nombre 1-100]</t>
         </is>
       </c>
       <c r="R543" s="7" t="n"/>
@@ -38822,7 +38858,7 @@
       <c r="P544" s="7" t="n"/>
       <c r="Q544" s="6" t="inlineStr">
         <is>
-          <t>Clics [nombre] · Position moyenne [nombre 1-100]</t>
+          <t>Clics [nombre 0-] · Position moyenne [nombre 1-100]</t>
         </is>
       </c>
       <c r="R544" s="6" t="inlineStr">
@@ -39055,7 +39091,9 @@
           <t>nombre</t>
         </is>
       </c>
-      <c r="N547" s="7" t="n"/>
+      <c r="N547" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="O547" s="7" t="n"/>
       <c r="P547" s="7" t="n"/>
       <c r="Q547" s="7" t="n"/>
@@ -39331,7 +39369,9 @@
           <t>€</t>
         </is>
       </c>
-      <c r="N551" s="7" t="n"/>
+      <c r="N551" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="O551" s="7" t="n"/>
       <c r="P551" s="7" t="n"/>
       <c r="Q551" s="7" t="n"/>
@@ -39402,7 +39442,7 @@
       <c r="P552" s="7" t="n"/>
       <c r="Q552" s="6" t="inlineStr">
         <is>
-          <t>Clics par mois [nombre] · Demandes par mois [nombre]</t>
+          <t>Clics par mois [nombre 0-] · Demandes par mois [nombre 0-]</t>
         </is>
       </c>
       <c r="R552" s="7" t="n"/>
@@ -39550,7 +39590,7 @@
       <c r="P554" s="7" t="n"/>
       <c r="Q554" s="6" t="inlineStr">
         <is>
-          <t>Clics [nombre] · Dépense [€ 0-] · Demandes [nombre]</t>
+          <t>Clics [nombre 0-] · Dépense [€ 0-] · Demandes [nombre 0-]</t>
         </is>
       </c>
       <c r="R554" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Vérification du questionnaire : règles d'affichage dans le navigateur, sous-question de cadrage, cadrage effaçable, noms de lignes dans les erreurs, page 404
Plan et exécution du contrôle navigateur de chaque règle d'affichage dans les
deux sens (règle vraie, fausse, retour, actualisation, réponse gardée mais
inactive). Une sous-question de cadrage qui n'est plus posée ne compte plus
(D12 « en service ? »). Une question de cadrage répondue peut être effacée.
Un message d'erreur de tableau nomme la ligne comme l'écran. Page 404 en
français. Contrôles ajoutés : résultats, séparation des comptes, départs de
page, changements rapides, captures. Rapport et chiffres dans
docs/verification (exécution complète en cours).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VuMzauPSe4mKhw7WeK1nNo
</commit_message>
<xml_diff>
--- a/CAXE_Banque_Questions.xlsx
+++ b/CAXE_Banque_Questions.xlsx
@@ -39856,6 +39856,12 @@
           <t>%</t>
         </is>
       </c>
+      <c r="N558" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O558" s="6" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="559">
       <c r="A559" s="6" t="inlineStr">
@@ -39891,7 +39897,7 @@
       </c>
       <c r="Q559" s="6" t="inlineStr">
         <is>
-          <t>Heures de production [heures] · Heures possibles [heures]</t>
+          <t>Heures de production [heures 0-] · Heures possibles [heures 0-]</t>
         </is>
       </c>
     </row>
@@ -39931,6 +39937,12 @@
         <is>
           <t>%</t>
         </is>
+      </c>
+      <c r="N560" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O560" s="6" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="561">
@@ -39963,7 +39975,7 @@
       </c>
       <c r="Q561" s="6" t="inlineStr">
         <is>
-          <t>Délai total [jours] · Dont attente avant lancement [jours]</t>
+          <t>Délai total [jours 0-] · Dont attente avant lancement [jours 0-]</t>
         </is>
       </c>
     </row>
@@ -40003,6 +40015,9 @@
         <is>
           <t>heures</t>
         </is>
+      </c>
+      <c r="N562" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>